<commit_message>
fix: PLS en Streamlit Cloud (Python 3.11 y pandas 2.x)
Parche plspm path.loc, HTMT sin fill_diagonal read-only, y PLS solo con ítems del modelo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/examples/encuesta_restaurante_20.xlsx
+++ b/examples/encuesta_restaurante_20.xlsx
@@ -13584,19 +13584,19 @@
         <v>0.7921725591063287</v>
       </c>
       <c r="B2" t="n">
-        <v>0.8168099880076392</v>
+        <v>0.8107550421498084</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06320842205427568</v>
+        <v>0.05476141716877299</v>
       </c>
       <c r="D2" t="n">
-        <v>0.698646048263632</v>
+        <v>0.7024179455696645</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9261996276939153</v>
+        <v>0.9069725397762469</v>
       </c>
       <c r="F2" t="n">
-        <v>12.5327058224315</v>
+        <v>14.46588857744272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>